<commit_message>
Cambio de tipo de archivo de empleados.xlsx
</commit_message>
<xml_diff>
--- a/XSD2025_2026/DAM/empladosEmpresa.xlsx
+++ b/XSD2025_2026/DAM/empladosEmpresa.xlsx
@@ -1,12 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://campuscamarasevilla-my.sharepoint.com/personal/willman_acosta_campuscamarasevilla_onmicrosoft_com/Documents/Documentos/2025_2026/LDM/LMSGI/XSD2025_2026/DAM/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_E75745071E43C9D64BBEDE4A7C9DA1DB7041F65F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EFC4ABA-7E3A-4FBE-9F27-44A22E164EDD}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Hoja 1" sheetId="1" r:id="rId5"/>
+    <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -34,21 +56,23 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -59,7 +83,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -69,43 +93,45 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -295,20 +321,24 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="5" max="5" width="14.88"/>
+    <col min="5" max="5" width="14.85546875" customWidth="1"/>
+    <col min="6" max="6" width="26.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -328,368 +358,368 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IMPORTXML(""https://raw.githubusercontent.com/willeusa/LMSGI/refs/heads/main/XSD2025_2026/DAM/empleados.xml"", ""//empleado"")"),"Ana")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("IMPORTXML(""https://raw.githubusercontent.com/willeusa/LMSGI/refs/heads/main/XSD2025_2026/DAM/empleados.xml"", ""//empleado"")"),"Ana")</f>
         <v>Ana</v>
       </c>
       <c r="C2" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"García")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"García")</f>
         <v>García</v>
       </c>
-      <c r="D2" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),30.0)</f>
+      <c r="D2" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),30)</f>
         <v>30</v>
       </c>
       <c r="E2" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ventas")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ventas")</f>
         <v>Ventas</v>
       </c>
       <c r="F2" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ejecutivo de ventas")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ejecutivo de ventas")</f>
         <v>Ejecutivo de ventas</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="B3" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Luis")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Luis")</f>
         <v>Luis</v>
       </c>
       <c r="C3" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Rodríguez")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Rodríguez")</f>
         <v>Rodríguez</v>
       </c>
-      <c r="D3" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),45.0)</f>
+      <c r="D3" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),45)</f>
         <v>45</v>
       </c>
       <c r="E3" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Finanzas")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Finanzas")</f>
         <v>Finanzas</v>
       </c>
       <c r="F3" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Analista financiero")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Analista financiero")</f>
         <v>Analista financiero</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="B4" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"María")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"María")</f>
         <v>María</v>
       </c>
       <c r="C4" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"López")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"López")</f>
         <v>López</v>
       </c>
-      <c r="D4" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),28.0)</f>
+      <c r="D4" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),28)</f>
         <v>28</v>
       </c>
       <c r="E4" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Marketing")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Marketing")</f>
         <v>Marketing</v>
       </c>
       <c r="F4" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Especialista en redes sociales")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Especialista en redes sociales")</f>
         <v>Especialista en redes sociales</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="B5" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Carlos")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Carlos")</f>
         <v>Carlos</v>
       </c>
       <c r="C5" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ruiz")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ruiz")</f>
         <v>Ruiz</v>
       </c>
-      <c r="D5" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),34.0)</f>
+      <c r="D5" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),34)</f>
         <v>34</v>
       </c>
       <c r="E5" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sistemas")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sistemas")</f>
         <v>Sistemas</v>
       </c>
       <c r="F5" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Administrador de redes")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Administrador de redes")</f>
         <v>Administrador de redes</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="B6" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Elena")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Elena")</f>
         <v>Elena</v>
       </c>
       <c r="C6" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sanz")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sanz")</f>
         <v>Sanz</v>
       </c>
-      <c r="D6" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),41.0)</f>
+      <c r="D6" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),41)</f>
         <v>41</v>
       </c>
       <c r="E6" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"RRHH")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"RRHH")</f>
         <v>RRHH</v>
       </c>
       <c r="F6" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Responsable de talento")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Responsable de talento")</f>
         <v>Responsable de talento</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="B7" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Javier")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Javier")</f>
         <v>Javier</v>
       </c>
       <c r="C7" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Martín")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Martín")</f>
         <v>Martín</v>
       </c>
-      <c r="D7" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),29.0)</f>
+      <c r="D7" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),29)</f>
         <v>29</v>
       </c>
       <c r="E7" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ventas")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ventas")</f>
         <v>Ventas</v>
       </c>
       <c r="F7" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Comercial junior")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Comercial junior")</f>
         <v>Comercial junior</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="B8" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sofía")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sofía")</f>
         <v>Sofía</v>
       </c>
       <c r="C8" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Castro")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Castro")</f>
         <v>Castro</v>
       </c>
-      <c r="D8" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),37.0)</f>
+      <c r="D8" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),37)</f>
         <v>37</v>
       </c>
       <c r="E8" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"I+D")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"I+D")</f>
         <v>I+D</v>
       </c>
       <c r="F8" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ingeniera de software")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ingeniera de software")</f>
         <v>Ingeniera de software</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="B9" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pablo")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pablo")</f>
         <v>Pablo</v>
       </c>
       <c r="C9" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Gómez")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Gómez")</f>
         <v>Gómez</v>
       </c>
-      <c r="D9" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),50.0)</f>
+      <c r="D9" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),50)</f>
         <v>50</v>
       </c>
       <c r="E9" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Logística")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Logística")</f>
         <v>Logística</v>
       </c>
       <c r="F9" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jefe de almacén")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jefe de almacén")</f>
         <v>Jefe de almacén</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="B10" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Lucía")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Lucía")</f>
         <v>Lucía</v>
       </c>
       <c r="C10" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Fernández")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Fernández")</f>
         <v>Fernández</v>
       </c>
-      <c r="D10" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),26.0)</f>
+      <c r="D10" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),26)</f>
         <v>26</v>
       </c>
       <c r="E10" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Marketing")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Marketing")</f>
         <v>Marketing</v>
       </c>
       <c r="F10" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Diseñadora gráfica")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Diseñadora gráfica")</f>
         <v>Diseñadora gráfica</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B11" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Antonio")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Antonio")</f>
         <v>Antonio</v>
       </c>
       <c r="C11" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Vázquez")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Vázquez")</f>
         <v>Vázquez</v>
       </c>
-      <c r="D11" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),44.0)</f>
+      <c r="D11" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),44)</f>
         <v>44</v>
       </c>
       <c r="E11" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Finanzas")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Finanzas")</f>
         <v>Finanzas</v>
       </c>
       <c r="F11" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Contable")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Contable")</f>
         <v>Contable</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="B12" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Marta")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Marta")</f>
         <v>Marta</v>
       </c>
       <c r="C12" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jiménez")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jiménez")</f>
         <v>Jiménez</v>
       </c>
-      <c r="D12" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),32.0)</f>
+      <c r="D12" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),32)</f>
         <v>32</v>
       </c>
       <c r="E12" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sistemas")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sistemas")</f>
         <v>Sistemas</v>
       </c>
       <c r="F12" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Analista de datos")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Analista de datos")</f>
         <v>Analista de datos</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="B13" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Raúl")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Raúl")</f>
         <v>Raúl</v>
       </c>
       <c r="C13" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pérez")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pérez")</f>
         <v>Pérez</v>
       </c>
-      <c r="D13" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),39.0)</f>
+      <c r="D13" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),39)</f>
         <v>39</v>
       </c>
       <c r="E13" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Dirección")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Dirección")</f>
         <v>Dirección</v>
       </c>
       <c r="F13" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Director general")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Director general")</f>
         <v>Director general</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>13.0</v>
+        <v>13</v>
       </c>
       <c r="B14" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Isabel")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Isabel")</f>
         <v>Isabel</v>
       </c>
       <c r="C14" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Blanco")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Blanco")</f>
         <v>Blanco</v>
       </c>
-      <c r="D14" s="4">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),31.0)</f>
+      <c r="D14" s="2">
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),31)</f>
         <v>31</v>
       </c>
       <c r="E14" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Atención al Cliente")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Atención al Cliente")</f>
         <v>Atención al Cliente</v>
       </c>
       <c r="F14" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Soporte técnico")</f>
+        <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Soporte técnico")</f>
         <v>Soporte técnico</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="str">
-        <f t="shared" ref="A15:A20" si="1">IF(B15="TRUE",1+A14,"")</f>
+        <f t="shared" ref="A15:A20" si="0">IF(B15="TRUE",1+A14,"")</f>
         <v/>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>